<commit_message>
chore(calendrier): xlsx + pdf + rapport [2026-10-10 15:51] UTC
</commit_message>
<xml_diff>
--- a/calendrier-paroissial/Calendrier_paroissial_2026-2027.xlsx
+++ b/calendrier-paroissial/Calendrier_paroissial_2026-2027.xlsx
@@ -2882,7 +2882,7 @@
       </c>
       <c r="Q26" s="22" t="n"/>
       <c r="S26" s="23" t="n"/>
-      <c r="T26" s="24" t="n"/>
+      <c r="T26" s="26" t="n"/>
       <c r="U26" s="22" t="n"/>
       <c r="W26" s="23" t="n"/>
       <c r="X26" s="27" t="n"/>
@@ -2933,7 +2933,11 @@
       <c r="Q27" s="29" t="n"/>
       <c r="R27" s="30" t="n"/>
       <c r="S27" s="31" t="n"/>
-      <c r="T27" s="26" t="n"/>
+      <c r="T27" s="16" t="inlineStr">
+        <is>
+          <t>Rencontre CCN + Kion</t>
+        </is>
+      </c>
       <c r="U27" s="29" t="n"/>
       <c r="V27" s="30" t="n"/>
       <c r="W27" s="31" t="n"/>
@@ -6071,7 +6075,11 @@
         <v>22</v>
       </c>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="19" t="n"/>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Rentrée District CCN + Kion</t>
+        </is>
+      </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
           <t>J</t>
@@ -6202,7 +6210,7 @@
     <row r="68" ht="20.1" customHeight="1">
       <c r="A68" s="22" t="n"/>
       <c r="C68" s="23" t="n"/>
-      <c r="D68" s="27" t="n"/>
+      <c r="D68" s="24" t="n"/>
       <c r="E68" s="22" t="n"/>
       <c r="G68" s="25" t="n"/>
       <c r="H68" s="24" t="n"/>
@@ -6245,7 +6253,7 @@
       <c r="A69" s="29" t="n"/>
       <c r="B69" s="30" t="n"/>
       <c r="C69" s="31" t="n"/>
-      <c r="D69" s="33" t="n"/>
+      <c r="D69" s="26" t="n"/>
       <c r="E69" s="29" t="n"/>
       <c r="F69" s="30" t="n"/>
       <c r="G69" s="32" t="n"/>
@@ -7743,7 +7751,7 @@
         <v>29</v>
       </c>
       <c r="AA88" s="7" t="n"/>
-      <c r="AB88" s="20" t="inlineStr">
+      <c r="AB88" s="17" t="inlineStr">
         <is>
           <t>Lundi de Pâques</t>
         </is>
@@ -7825,7 +7833,11 @@
       <c r="T89" s="27" t="n"/>
       <c r="Y89" s="22" t="n"/>
       <c r="AA89" s="23" t="n"/>
-      <c r="AB89" s="24" t="n"/>
+      <c r="AB89" s="16" t="inlineStr">
+        <is>
+          <t>Lundi de Pâques CCN + Kion + Cana</t>
+        </is>
+      </c>
       <c r="AC89" s="22" t="n"/>
       <c r="AE89" s="25" t="n"/>
       <c r="AF89" s="27" t="n"/>
@@ -7866,7 +7878,7 @@
       <c r="Y90" s="29" t="n"/>
       <c r="Z90" s="30" t="n"/>
       <c r="AA90" s="31" t="n"/>
-      <c r="AB90" s="26" t="n"/>
+      <c r="AB90" s="33" t="n"/>
       <c r="AC90" s="29" t="n"/>
       <c r="AD90" s="30" t="n"/>
       <c r="AE90" s="32" t="n"/>
@@ -8559,6 +8571,7 @@
     <mergeCell ref="AS19:AS21"/>
     <mergeCell ref="Z88:Z90"/>
     <mergeCell ref="F67:F69"/>
+    <mergeCell ref="D67:D69"/>
     <mergeCell ref="F82:F84"/>
     <mergeCell ref="AP16:AP18"/>
     <mergeCell ref="A79:A81"/>
@@ -8693,6 +8706,7 @@
     <mergeCell ref="Q85:Q87"/>
     <mergeCell ref="E61:E63"/>
     <mergeCell ref="AT4:AT6"/>
+    <mergeCell ref="T19:T26"/>
     <mergeCell ref="AO43:AO45"/>
     <mergeCell ref="AC19:AC21"/>
     <mergeCell ref="D4:D6"/>
@@ -8777,7 +8791,6 @@
     <mergeCell ref="M64:M66"/>
     <mergeCell ref="Q28:Q30"/>
     <mergeCell ref="AR43:AR45"/>
-    <mergeCell ref="AB88:AB90"/>
     <mergeCell ref="V64:V66"/>
     <mergeCell ref="B43:B45"/>
     <mergeCell ref="F7:F9"/>
@@ -9040,7 +9053,6 @@
     <mergeCell ref="AK91:AK93"/>
     <mergeCell ref="AO49:AO51"/>
     <mergeCell ref="P38:P40"/>
-    <mergeCell ref="T19:T27"/>
     <mergeCell ref="N70:N72"/>
     <mergeCell ref="AH13:AH15"/>
     <mergeCell ref="AL46:AL48"/>

</xml_diff>